<commit_message>
update git commit log
</commit_message>
<xml_diff>
--- a/HW01_Test_Cases_Checklist_Summary.xlsx
+++ b/HW01_Test_Cases_Checklist_Summary.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" r:id="Rcc60f1f1452d4df2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ca kiểm thử" sheetId="2" r:id="R1bdddef905f54a8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Link video" sheetId="3" r:id="R483524aeb8da44b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nhật ký defect" sheetId="4" r:id="R13053d512d4b4b79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh sách kiểm tra" sheetId="5" r:id="R375e7e1e344c48de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Truy vết" sheetId="6" r:id="R8ba103e8295e43bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tự chấm" sheetId="7" r:id="Red43c0211cc84572"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" r:id="R941c075fd7234261"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ca kiểm thử" sheetId="2" r:id="Rdd0f8890510d460e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Link video" sheetId="3" r:id="R656ad137bb6f496e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nhật ký defect" sheetId="4" r:id="Rb90b837485f143c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh sách kiểm tra" sheetId="5" r:id="R1e57700e842c4e5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Truy vết" sheetId="6" r:id="Re9ca6670420744ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tự chấm" sheetId="7" r:id="R6744ad18a8d44680"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1514,8 +1514,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TongQuanTable" displayName="TongQuanTable" ref="A1:D11" totalsRowShown="0">
-  <x:autoFilter ref="A1:D11"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TongQuanTable" displayName="TongQuanTable" ref="A1:D12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:D12"/>
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Hạng mục"/>
     <x:tableColumn id="2" name="Giá trị"/>
@@ -1595,8 +1595,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ChecklistTable" displayName="ChecklistTable" ref="A1:D18" totalsRowShown="0">
-  <x:autoFilter ref="A1:D18"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ChecklistTable" displayName="ChecklistTable" ref="A1:D19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:D19"/>
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Hạng mục checklist"/>
     <x:tableColumn id="2" name="Trạng thái"/>
@@ -1608,8 +1608,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TraceabilityTable" displayName="TraceabilityTable" ref="A1:D18" totalsRowShown="0">
-  <x:autoFilter ref="A1:D18"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TraceabilityTable" displayName="TraceabilityTable" ref="A1:D19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:D19"/>
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Yêu cầu / Artifact"/>
     <x:tableColumn id="2" name="Evidence/File"/>
@@ -1947,10 +1947,24 @@
         <x:v>Đạt; 10 video &lt;=60 giây, có giọng nói và ở chế độ Unlisted</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>Git commit log và ảnh Terminal</x:v>
+      </x:c>
+      <x:c r="B12" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>Có lịch sử commit</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>Đạt; GIT_COMMIT_LOG.md và 7 ảnh Terminal</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb093408195f64135"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc148ba956ecf4d9b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2977,30 +2991,30 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="R4889516b855c464d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="Re260230cbfe64ae2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="R10e198e4de824719"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="Rfa0589f8ca1344c7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="R939cb046286847f7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="R5c19604c07d54de3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="Rebe4a5cb777d4914"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="R92077fe4a99f463b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="Rd2bc0f24022a464b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="R3e4cd6aa30564c45"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="Rb60f76b7d3f44dfa"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="R0e649e5e38d14d2c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="R84da43c44f294de4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="Raa7c5f1c4c3e4fa0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="Ra118bc61f6ea41dc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="Re857a85c97af4269"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="Rd150d567d2bf40cf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="Ra150db120caf4dee"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="R65864619e2d345db"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="Rfad4c00604c54790"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="R06df334d40c34962"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="Rbab6b9d3d03f4c1b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="R4bd20fe2276d4d44"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="R3defabc48ff34ae2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="R7456d9777edf4f73"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="Rf3bad5596bc44f32"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="R73b1a8a26c5345e6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="R805e06753c64409a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="R9a260b9b4ba64d1c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="R982e1320c3ec40a6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="Rb4ef8900535a47b4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="R03391e23cdff4a07"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="Rd4f155ded63c4bee"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="Rdd42e53178034e4c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="R7871531f6d484928"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="R3f839963f9744a64"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="R05b7303c64b846b8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="R1103dcebf775433c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="Rbf9fcaebb70248f5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="Rdf36516636354e6c"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raee865f5c0734889"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3739f7d45cdd488e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3281,16 +3295,16 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="R93b202c4f2d649ec"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="Raa35269576d84e4b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="Rae7d5aec175d4506"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="R08faa16bbc004cd4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="R59b3a707fd964254"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="R78d8c4d2200e4d6b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="Rb226d57362264122"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="Rbab0dace018c48a0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="R385c504a6ef644ca"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="Rbe652de952eb4ea7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="R3131899994414097"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="Rdb4d592632d7416e"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R426bc8d5afc84dfb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cbbb1144ab7449c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3568,15 +3582,15 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="R3cf759b155f146bc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="Rc391333bd7474742"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="R9cdcdb714711499a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="R7e5c7bbbdb9d42a4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="R2e11a41bbc4445f9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="R4ed2767aabde4031"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="R7bc82f725038408d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="Rbbcce8ff17b54e85"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="R16f86c3b91cb4c7d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="Rbbc468a071a64997"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94bacab5e67b4f73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref3458fc750e4ba5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3842,6 +3856,20 @@
         <x:v>324</x:v>
       </x:c>
     </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>Git commit log và ảnh chụp Terminal</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>Đã hoàn thành</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>Sinh viên</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>GIT_COMMIT_LOG.md; 7 ảnh tại evidence/git_commit_log/</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="B2:B18">
     <x:cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Đã hoàn thành"/>
@@ -3853,11 +3881,11 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="R8119f3d0edb3430f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="Rb8ededf35fa0446c"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc124b0776cc54742"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2497a83e9d624f34"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4116,13 +4144,27 @@
         <x:v>Repository đã đặt Public và có thể truy cập mà không cần đăng nhập</x:v>
       </x:c>
     </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>Git commit log</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>GIT_COMMIT_LOG.md và evidence/git_commit_log/</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>Đã có</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>20 commit được minh chứng bằng 7 ảnh Terminal</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="Rcd0a8b1c31434463"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="Rf3c5b756638241ca"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15d2c4feb8374c67"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdea571ee8b494bb7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4254,7 +4296,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E7" s="17" t="str">
-        <x:v>AI-05 bằng Markdown/PDF đã có; 5 GitHub Issues và ảnh tổng quan đã bổ sung; còn cần screenshot chứng minh AI bỏ sót edge case</x:v>
+        <x:v>AI-05, 5 GitHub Issues, ảnh Issues, Git commit log và 7 ảnh Terminal đã được bổ sung</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" customHeight="1">
@@ -4274,7 +4316,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R417c792936184c53"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf963f09ba664016"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>